<commit_message>
Enrich top-100 LinkedIn pages via Apollo.io + web cross-check
Ran Apollo bulk organization enrichment on all 90 company domains and
merged with the prior web-search results. Combined coverage is now 68 of
100 (Apollo matched 61, web search 54). Apollo filled 14 gaps web search
missed (incl. Fabbro Hnos, Funcke, and CJK/Hebrew-slug pages). Where the
sources disagreed, kept the location-specific web-verified URL; used
Apollo to fill gaps; flagged 2 Apollo domain-matches as verify.

- World_distributor_Gearboxes_LinkedIn.xlsx (column U updated to 68 pages)
- linkedin_apollo_vs_web.csv (side-by-side Apollo vs web for all 100)
- README.md (refreshed summary + tables)

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01LnG7g34kHynD55ncWN8uhz
</commit_message>
<xml_diff>
--- a/linkedin-research/World_distributor_Gearboxes_LinkedIn.xlsx
+++ b/linkedin-research/World_distributor_Gearboxes_LinkedIn.xlsx
@@ -845,6 +845,11 @@
           <t>General industrial</t>
         </is>
       </c>
+      <c r="U4" t="inlineStr">
+        <is>
+          <t>linkedin.com/company/fabbro-hnos-saic</t>
+        </is>
+      </c>
       <c r="Y4" s="2" t="inlineStr">
         <is>
           <t>57 yrs; regional exporter</t>
@@ -2466,6 +2471,11 @@
           <t>General industrial</t>
         </is>
       </c>
+      <c r="U26" t="inlineStr">
+        <is>
+          <t>linkedin.com/company/funckeacoplamentos</t>
+        </is>
+      </c>
       <c r="Y26" s="2" t="n"/>
       <c r="Z26" t="inlineStr">
         <is>
@@ -3430,6 +3440,11 @@
           <t>Material handling, lifting</t>
         </is>
       </c>
+      <c r="U39" t="inlineStr">
+        <is>
+          <t>linkedin.com/company/engineered-lifting-systems-llc</t>
+        </is>
+      </c>
       <c r="Y39" s="2" t="inlineStr">
         <is>
           <t>NORD parts distributor N. America</t>
@@ -4782,6 +4797,11 @@
           <t>General industrial</t>
         </is>
       </c>
+      <c r="U57" t="inlineStr">
+        <is>
+          <t>linkedin.com/company/上海欧传传动机械有限公司</t>
+        </is>
+      </c>
       <c r="Y57" s="2" t="inlineStr">
         <is>
           <t>Makes replacements for EU brands</t>
@@ -8589,6 +8609,11 @@
           <t>General industrial</t>
         </is>
       </c>
+      <c r="U109" t="inlineStr">
+        <is>
+          <t>linkedin.com/company/tramec-riduttori</t>
+        </is>
+      </c>
       <c r="Y109" s="2" t="inlineStr">
         <is>
           <t>Tramec German subsidiary</t>
@@ -11708,6 +11733,11 @@
           <t>General industrial</t>
         </is>
       </c>
+      <c r="U151" t="inlineStr">
+        <is>
+          <t>linkedin.com/company/cv-multi-mas</t>
+        </is>
+      </c>
       <c r="Y151" s="2" t="inlineStr">
         <is>
           <t>Official SEW distributor Indonesia</t>
@@ -12951,6 +12981,11 @@
           <t>General industrial</t>
         </is>
       </c>
+      <c r="U168" t="inlineStr">
+        <is>
+          <t>linkedin.com/company/לירז-הנדסה-בע</t>
+        </is>
+      </c>
       <c r="Y168" s="2" t="n"/>
       <c r="Z168" t="inlineStr">
         <is>
@@ -14750,6 +14785,11 @@
           <t>General industrial</t>
         </is>
       </c>
+      <c r="U193" t="inlineStr">
+        <is>
+          <t>linkedin.com/company/高津伝動精機株式会社</t>
+        </is>
+      </c>
       <c r="Y193" s="2" t="inlineStr">
         <is>
           <t>SEW sales agent in Japan</t>
@@ -17631,6 +17671,11 @@
           <t>General industrial</t>
         </is>
       </c>
+      <c r="U232" t="inlineStr">
+        <is>
+          <t>linkedin.com/company/ntpiofficial</t>
+        </is>
+      </c>
       <c r="Y232" s="2" t="inlineStr">
         <is>
           <t>Unit 719 Globe Telecom Plaza 2, Mandaluyong</t>
@@ -18798,6 +18843,11 @@
           <t>General industrial</t>
         </is>
       </c>
+      <c r="U248" t="inlineStr">
+        <is>
+          <t>linkedin.com/company/lemus-enterprises-the-online-electrical-store</t>
+        </is>
+      </c>
       <c r="Y248" s="2" t="inlineStr">
         <is>
           <t>Multi-country GCC/Africa reach</t>
@@ -19024,6 +19074,11 @@
           <t>Industrial</t>
         </is>
       </c>
+      <c r="U251" t="inlineStr">
+        <is>
+          <t>linkedin.com/company/casisenegal</t>
+        </is>
+      </c>
       <c r="Y251" s="2" t="inlineStr">
         <is>
           <t>Industrial transmission specialist</t>
@@ -19250,6 +19305,11 @@
           <t>General industrial</t>
         </is>
       </c>
+      <c r="U254" t="inlineStr">
+        <is>
+          <t>linkedin.com/company/plant-&amp;-mill-motion-control-sdn-bhd</t>
+        </is>
+      </c>
       <c r="Y254" s="2" t="inlineStr">
         <is>
           <t>Regional SE-Asia coverage</t>
@@ -29768,6 +29828,11 @@
           <t>General industrial</t>
         </is>
       </c>
+      <c r="U398" t="inlineStr">
+        <is>
+          <t>linkedin.com/company/daikinhnam</t>
+        </is>
+      </c>
       <c r="Y398" s="2" t="inlineStr">
         <is>
           <t>2 DT743, An Phu, Binh Duong</t>
@@ -29916,6 +29981,11 @@
       <c r="S400" t="inlineStr">
         <is>
           <t>Mining, industrial</t>
+        </is>
+      </c>
+      <c r="U400" t="inlineStr">
+        <is>
+          <t>linkedin.com/company/powerdrive-transmission-suppliers</t>
         </is>
       </c>
       <c r="Y400" s="2" t="n"/>

</xml_diff>